<commit_message>
Include new venues in growth template
</commit_message>
<xml_diff>
--- a/templates/03_Venue_Details_Template_v2.xlsx
+++ b/templates/03_Venue_Details_Template_v2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Venues" sheetId="1" r:id="R36d3928c1ea4492e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ramp Up" sheetId="2" r:id="R50e6934ada3042bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly Growth" sheetId="3" r:id="R96d40ae65ee7466a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="New Venues" sheetId="4" r:id="Rb3e5c40c8e854fd5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Venues" sheetId="1" r:id="R8d29e6d34200450f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ramp Up" sheetId="2" r:id="R80f2f303ba22423c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly Growth" sheetId="3" r:id="R9c9d39a54fd5433a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="New Venues" sheetId="4" r:id="R4f7666364a9c4031"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -10569,6 +10569,1009 @@
         <x:v>3</x:v>
       </x:c>
     </x:row>
+    <x:row r="71">
+      <x:c r="A71" s="7" t="str">
+        <x:v>Yo-Chi New Venue 01</x:v>
+      </x:c>
+      <x:c r="B71" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C71" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D71" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E71" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F71" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G71" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H71" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I71" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="J71" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="K71" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L71" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="M71" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="N71" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O71" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="P71" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="Q71" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="R71" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="S71" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72">
+      <x:c r="A72" s="7" t="str">
+        <x:v>Yo-Chi New Venue 02</x:v>
+      </x:c>
+      <x:c r="B72" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C72" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D72" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E72" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F72" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G72" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H72" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I72" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="J72" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="K72" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L72" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="M72" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="N72" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O72" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="P72" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="Q72" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="R72" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="S72" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73">
+      <x:c r="A73" s="7" t="str">
+        <x:v>Yo-Chi New Venue 03</x:v>
+      </x:c>
+      <x:c r="B73" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C73" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D73" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E73" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F73" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G73" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H73" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I73" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="J73" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="K73" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L73" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="M73" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="N73" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O73" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="P73" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="Q73" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="R73" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="S73" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74">
+      <x:c r="A74" s="7" t="str">
+        <x:v>Yo-Chi New Venue 04</x:v>
+      </x:c>
+      <x:c r="B74" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C74" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D74" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E74" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F74" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G74" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H74" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I74" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="J74" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="K74" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L74" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="M74" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="N74" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O74" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="P74" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="Q74" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="R74" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="S74" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75">
+      <x:c r="A75" s="7" t="str">
+        <x:v>Yo-Chi New Venue 05</x:v>
+      </x:c>
+      <x:c r="B75" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C75" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D75" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E75" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F75" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G75" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H75" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I75" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="J75" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="K75" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L75" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="M75" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="N75" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O75" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="P75" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="Q75" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="R75" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="S75" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76">
+      <x:c r="A76" s="7" t="str">
+        <x:v>Yo-Chi New Venue 06</x:v>
+      </x:c>
+      <x:c r="B76" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C76" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D76" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E76" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F76" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G76" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H76" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I76" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="J76" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="K76" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L76" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="M76" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="N76" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O76" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="P76" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="Q76" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="R76" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="S76" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77">
+      <x:c r="A77" s="7" t="str">
+        <x:v>Yo-Chi New Venue 07</x:v>
+      </x:c>
+      <x:c r="B77" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C77" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D77" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E77" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F77" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G77" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H77" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I77" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="J77" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="K77" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L77" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="M77" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="N77" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O77" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="P77" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="Q77" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="R77" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="S77" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78">
+      <x:c r="A78" s="7" t="str">
+        <x:v>Yo-Chi New Venue 08</x:v>
+      </x:c>
+      <x:c r="B78" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C78" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D78" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E78" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F78" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G78" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H78" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I78" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="J78" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="K78" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L78" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="M78" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="N78" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O78" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="P78" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="Q78" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="R78" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="S78" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="79">
+      <x:c r="A79" s="7" t="str">
+        <x:v>Yo-Chi New Venue 09</x:v>
+      </x:c>
+      <x:c r="B79" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C79" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D79" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E79" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F79" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G79" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H79" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I79" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="J79" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="K79" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L79" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="M79" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="N79" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O79" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="P79" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="Q79" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="R79" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="S79" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80">
+      <x:c r="A80" s="7" t="str">
+        <x:v>Yo-Chi New Venue 10</x:v>
+      </x:c>
+      <x:c r="B80" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C80" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D80" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E80" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F80" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G80" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H80" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I80" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="J80" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="K80" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L80" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="M80" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="N80" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O80" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="P80" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="Q80" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="R80" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="S80" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="81">
+      <x:c r="A81" s="7" t="str">
+        <x:v>Yo-Chi New Venue 11</x:v>
+      </x:c>
+      <x:c r="B81" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C81" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D81" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E81" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F81" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G81" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H81" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I81" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="J81" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="K81" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L81" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="M81" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="N81" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O81" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="P81" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="Q81" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="R81" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="S81" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="82">
+      <x:c r="A82" s="7" t="str">
+        <x:v>Yo-Chi New Venue 12</x:v>
+      </x:c>
+      <x:c r="B82" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C82" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D82" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E82" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F82" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G82" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H82" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I82" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="J82" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="K82" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L82" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="M82" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="N82" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O82" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="P82" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="Q82" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="R82" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="S82" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="83">
+      <x:c r="A83" s="7" t="str">
+        <x:v>Yo-Chi New Venue 13</x:v>
+      </x:c>
+      <x:c r="B83" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C83" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D83" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E83" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F83" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G83" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H83" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I83" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="J83" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="K83" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L83" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="M83" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="N83" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O83" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="P83" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="Q83" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="R83" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="S83" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="84">
+      <x:c r="A84" s="7" t="str">
+        <x:v>Yo-Chi New Venue 14</x:v>
+      </x:c>
+      <x:c r="B84" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C84" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D84" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E84" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F84" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G84" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H84" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I84" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="J84" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="K84" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L84" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="M84" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="N84" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O84" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="P84" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="Q84" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="R84" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="S84" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="85">
+      <x:c r="A85" s="7" t="str">
+        <x:v>Yo-Chi New Venue 15</x:v>
+      </x:c>
+      <x:c r="B85" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C85" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D85" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E85" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F85" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G85" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H85" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I85" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="J85" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="K85" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L85" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="M85" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="N85" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O85" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="P85" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="Q85" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="R85" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="S85" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="86">
+      <x:c r="A86" s="7" t="str">
+        <x:v>Yo-Chi New Venue 16</x:v>
+      </x:c>
+      <x:c r="B86" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C86" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D86" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E86" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F86" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G86" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H86" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I86" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="J86" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="K86" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L86" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="M86" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="N86" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O86" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="P86" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="Q86" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="R86" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="S86" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="87">
+      <x:c r="A87" s="7" t="str">
+        <x:v>Yo-Chi New Venue 17</x:v>
+      </x:c>
+      <x:c r="B87" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C87" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D87" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E87" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F87" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G87" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H87" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I87" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="J87" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="K87" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L87" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="M87" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="N87" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O87" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="P87" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="Q87" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="R87" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="S87" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>